<commit_message>
Use template table for Excel export and update resources
Update Graficos.cs to export data into an existing Excel table (TabelaDados): clear the table data range, InsertData starting at row 2, resize the table to the new data range, adjust columns, save and open the workbook, and improve success/error messages. Add new Rel.xlsx and reorganize the RelatorioConsumos.xlsx EmbeddedResource entry in PEPIDI.csproj. Also include incidental updates to Visual Studio layout/metadata files, assembly informational version and source-link references (build artifacts and .vs cache changes).
</commit_message>
<xml_diff>
--- a/PEPIDI-0.5/RelatorioConsumos.xlsx
+++ b/PEPIDI-0.5/RelatorioConsumos.xlsx
@@ -8,20 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bruno.oliveira\Desktop\PEPIDI-0.5\PEPIDI-0.5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C411BDC9-C1F8-4E66-9E5E-A5E7755B2E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61EBFB6B-FD85-4EDE-8E04-3360A4BBF12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5039FA72-8519-4402-BA42-7581F30CB7F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4072F3FA-7EF8-4191-9F23-D9CB75462A9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="TabelaDados">Dados!$A:$J</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId3"/>
+    <pivotCache cacheId="19" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
   <si>
     <t>Data</t>
   </si>
@@ -72,6 +69,24 @@
   <si>
     <t>TotalGasto</t>
   </si>
+  <si>
+    <t>Rótulos de Linha</t>
+  </si>
+  <si>
+    <t>(em branco)</t>
+  </si>
+  <si>
+    <t>Total Geral</t>
+  </si>
+  <si>
+    <t>(Tudo)</t>
+  </si>
+  <si>
+    <t>Rótulos de Coluna</t>
+  </si>
+  <si>
+    <t>Soma de Quantidade</t>
+  </si>
 </sst>
 </file>
 
@@ -94,7 +109,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -102,148 +117,28 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFABABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFABABAB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFABABAB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFABABAB"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFABABAB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFABABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFABABAB"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFABABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFABABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFABABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFABABAB"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFABABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -270,17 +165,167 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[RelatorioConsumos.xlsx]Dashboard!Tabela Dinâmica1</c:name>
+    <c:name>[RelatorioConsumos.xlsx]Dashboard!TabelaDinâmica</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-PT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
     <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-PT"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$4:$C$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>(em branco)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Dashboard!$B$6:$B$9</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="1"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>(em branco)</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>(em branco)</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>(em branco)</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$6:$C$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-240A-483D-AD66-703440D92988}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -291,16 +336,17 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="826951888"/>
-        <c:axId val="826965808"/>
+        <c:axId val="1661593088"/>
+        <c:axId val="1661584448"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="826951888"/>
+        <c:axId val="1661593088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -337,7 +383,7 @@
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="826965808"/>
+        <c:crossAx val="1661584448"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -345,7 +391,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="826965808"/>
+        <c:axId val="1661584448"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -365,6 +411,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -395,7 +442,7 @@
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="826951888"/>
+        <c:crossAx val="1661593088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1045,23 +1092,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1885950</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Gráfico 1">
+        <xdr:cNvPr id="3" name="Gráfico 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2FFCC11D-A940-1747-E922-CC322EB5F9BF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4FA533BF-2A52-6AA8-DE43-8E19D1F0EB27}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1083,34 +1130,48 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Bruno Oliveira" refreshedDate="46120.651267013891" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{581299C6-927E-4E1E-A704-7AAA736DC0D7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Bruno Oliveira" refreshedDate="46122.421389814815" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{98C1E756-F3D1-461F-BAAA-2B2C7262A974}">
   <cacheSource type="worksheet">
     <worksheetSource name="TabelaDados"/>
   </cacheSource>
   <cacheFields count="10">
     <cacheField name="Data" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="NrFunc" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="NomeFuncionario" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Funcao" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Familia" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Modelo" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Tamanho" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Quantidade" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="PrecoUnitario" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
@@ -1130,14 +1191,14 @@
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="1">
   <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
     <m/>
     <m/>
   </r>
@@ -1145,20 +1206,106 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE52E9C3-09AD-4A60-9D24-6CB469FD1C04}" name="Tabela Dinâmica1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A1:C18" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{91F5E1FC-9DFB-4027-BAFA-63A1E31DF11D}" name="TabelaDinâmica" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="B4:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
+  <rowFields count="3">
+    <field x="0"/>
+    <field x="2"/>
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="1" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Soma de Quantidade" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1169,6 +1316,25 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{86B3A40B-17B9-471C-94A4-FAAE277FF014}" name="TabelaDados" displayName="TabelaDados" ref="A1:J2" totalsRowShown="0">
+  <autoFilter ref="A1:J2" xr:uid="{86B3A40B-17B9-471C-94A4-FAAE277FF014}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{BBEFF5B2-3172-40D3-9A24-7D12B258EA8A}" name="Data"/>
+    <tableColumn id="2" xr3:uid="{45F57951-21D9-418D-996A-6DD09A898A8D}" name="NrFunc"/>
+    <tableColumn id="3" xr3:uid="{D81E7836-F54E-4B74-95E8-3661D19029FD}" name="NomeFuncionario"/>
+    <tableColumn id="4" xr3:uid="{0587B062-162F-4BD0-90E7-05B8EBAF154D}" name="Funcao"/>
+    <tableColumn id="5" xr3:uid="{3C8C8960-EFA8-45BF-860D-7078091CB600}" name="Familia"/>
+    <tableColumn id="6" xr3:uid="{2EC100EB-DE9B-4B28-9A57-D6D20EDC3A78}" name="Modelo"/>
+    <tableColumn id="7" xr3:uid="{8245E0CB-15D6-4948-AF04-0C8BF4141D70}" name="Tamanho"/>
+    <tableColumn id="8" xr3:uid="{E75BD4F7-D914-4771-9807-3973B9806561}" name="Quantidade"/>
+    <tableColumn id="9" xr3:uid="{2473A3C4-9089-4F79-BF96-83F36EDC14E3}" name="PrecoUnitario"/>
+    <tableColumn id="10" xr3:uid="{4E2067A4-D39F-49A0-848B-EFA7EAF2A3C9}" name="TotalGasto"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1467,14 +1633,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CF1CC8C-C6AF-477C-A600-5DD5E58370A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1FE863-216B-46FD-B121-F7F94607EE87}">
   <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="52.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.28515625" customWidth="1"/>
-    <col min="5" max="10" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="57.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1510,115 +1682,85 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:J1">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83012DEC-872E-47EA-83E8-DDDE40769BA8}">
-  <dimension ref="A1:C18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF9E862-5C1F-4E07-A2BB-466FFB494875}">
+  <dimension ref="B1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="53.5703125" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="5" max="5" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3"/>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6"/>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="6"/>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="6"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="6"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="6"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>